<commit_message>
add testing for delete and insert cases
</commit_message>
<xml_diff>
--- a/expensesv2/data/Repository.xlsx
+++ b/expensesv2/data/Repository.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Formação\workspaceV2\expensesV2\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Formação\workspaceV2\expensesV2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2C3245-E96D-487C-AB6E-29DD7A79934E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55012EA5-A040-4086-82D5-8AD5B0196DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{14EC8011-9132-421C-BEF6-A483E0F6AAD9}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" activeTab="3" xr2:uid="{14EC8011-9132-421C-BEF6-A483E0F6AAD9}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>id</t>
   </si>
@@ -65,47 +65,16 @@
     <t>value</t>
   </si>
   <si>
-    <t>userid</t>
-  </si>
-  <si>
     <t>typeid</t>
-  </si>
-  <si>
-    <t>user_id</t>
-  </si>
-  <si>
-    <t>teste</t>
-  </si>
-  <si>
-    <t>user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pass </t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>1.4</t>
   </si>
   <si>
     <t>isRevenue</t>
   </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -475,13 +444,13 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -496,16 +465,16 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -520,20 +489,20 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s" s="0">
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
         <v>8</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -547,10 +516,10 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s" s="0">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -560,23 +529,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B2DFD334E6A3034F898C07A5B179AF82" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4b47bed1f976da8d6b40dd0f87550b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xmlns:ns4="e24bc939-ed6e-4865-8a4d-2519bddf4458" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="58236cf1faf4b8c1ff480fa16364175a" ns3:_="" ns4:_="">
     <xsd:import namespace="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
@@ -823,32 +775,24 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C863830A-F770-4763-8C49-E662B683E9A2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="e24bc939-ed6e-4865-8a4d-2519bddf4458"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A799487-F5F9-4CBB-B943-BF270F428C40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6C94329-D6A5-498C-999E-67C6D3CED00A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -865,4 +809,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A799487-F5F9-4CBB-B943-BF270F428C40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C863830A-F770-4763-8C49-E662B683E9A2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="e24bc939-ed6e-4865-8a4d-2519bddf4458"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
core done and User creation API done
</commit_message>
<xml_diff>
--- a/expensesv2/data/Repository.xlsx
+++ b/expensesv2/data/Repository.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Formação\workspaceV2\expensesV2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23A89B08-D58D-4125-9E38-6AF7E7284C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D93ED33-ABFE-4618-90EB-39E2665CEEAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{14EC8011-9132-421C-BEF6-A483E0F6AAD9}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
   <si>
     <t>id</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>isRevenue</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>admin</t>
   </si>
 </sst>
 </file>
@@ -440,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC48EE1E-E673-4715-ACB6-0AB99EDFE6FD}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -452,6 +458,17 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -529,23 +546,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B2DFD334E6A3034F898C07A5B179AF82" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4b47bed1f976da8d6b40dd0f87550b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xmlns:ns4="e24bc939-ed6e-4865-8a4d-2519bddf4458" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="58236cf1faf4b8c1ff480fa16364175a" ns3:_="" ns4:_="">
     <xsd:import namespace="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
@@ -792,32 +792,24 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C863830A-F770-4763-8C49-E662B683E9A2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="e24bc939-ed6e-4865-8a4d-2519bddf4458"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A799487-F5F9-4CBB-B943-BF270F428C40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6C94329-D6A5-498C-999E-67C6D3CED00A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -834,4 +826,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A799487-F5F9-4CBB-B943-BF270F428C40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C863830A-F770-4763-8C49-E662B683E9A2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="e24bc939-ed6e-4865-8a4d-2519bddf4458"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4d31cefb-fbe1-49e3-a6c0-31d87c931e3e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>